<commit_message>
Add a KPI-card style Dashboard sheet to the Excel report
New "Dashboard" sheet (set as the active sheet) mirrors the HTML
dashboard's layout inside Excel: title banner with embedded HAL
logo, 4 top-line KPI stat cards (shortfall alert, combined 40'RH
stock/booking/balance), a two-depot Detail table, AV/DMG remarks,
and RF Seasonal stat cards + current brand/size mix - all live
formulas referencing the TOTAL RH sheet, not hardcoded values.
apply_negatives_full.py now also colors negative AV-Balance cells
red on the Dashboard sheet (skipping the KPI cards, whose color is
set once by build_full.py).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_9-17.xlsx
+++ b/Stock_Daily_Reefer_9-17.xlsx
@@ -4,13 +4,14 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Control" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BookingRaw" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StockRaw" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TOTAL RH" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,6 +47,75 @@
       <sz val="9"/>
     </font>
     <font/>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C62828"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <color rgb="00808080"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000D3B12"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002A78D6"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00EB6834"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002A78D6"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00EB6834"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002A78D6"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00EB6834"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002A78D6"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00EB6834"/>
+      <sz val="10"/>
+    </font>
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -75,6 +145,47 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00808080"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00C62828"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A1A1A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00808080"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000D3B12"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002A78D6"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00EB6834"/>
       <sz val="11"/>
     </font>
     <font>
@@ -140,7 +251,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -162,92 +273,195 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -324,6 +538,39 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>17</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1619250" cy="400050"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5381,11 +5628,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="51">
         <f>C4-C5-C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="51">
         <f>D4-D5-D6-D7</f>
         <v/>
       </c>
@@ -5396,11 +5643,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C$4)&amp;" "&amp;CHOOSE(MONTH(Control!$C$4),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="51">
         <f>I4-I5-I6-I7</f>
         <v/>
       </c>
-      <c r="J8" s="31">
+      <c r="J8" s="51">
         <f>J4-J5-J6-J7</f>
         <v/>
       </c>
@@ -5479,11 +5726,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="51">
         <f>C8-C9</f>
         <v/>
       </c>
-      <c r="D10" s="32">
+      <c r="D10" s="52">
         <f>D8-D9</f>
         <v/>
       </c>
@@ -5494,11 +5741,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C5)&amp;" "&amp;CHOOSE(MONTH(Control!$C5),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I10" s="31">
+      <c r="I10" s="51">
         <f>I8-I9</f>
         <v/>
       </c>
-      <c r="J10" s="31">
+      <c r="J10" s="51">
         <f>J8-J9</f>
         <v/>
       </c>
@@ -5567,11 +5814,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="C12" s="31">
+      <c r="C12" s="51">
         <f>C10-C11</f>
         <v/>
       </c>
-      <c r="D12" s="32">
+      <c r="D12" s="52">
         <f>D10-D11</f>
         <v/>
       </c>
@@ -5582,11 +5829,11 @@
         <f>"AV Balance till "&amp;DAY(Control!$C6)&amp;" "&amp;CHOOSE(MONTH(Control!$C6),"JAN","FEB","MAR","APR","MAY","JUN","JUL","AUG","SEP","OCT","NOV","DEC")</f>
         <v/>
       </c>
-      <c r="I12" s="31">
+      <c r="I12" s="51">
         <f>I10-I11</f>
         <v/>
       </c>
-      <c r="J12" s="32">
+      <c r="J12" s="52">
         <f>J10-J11</f>
         <v/>
       </c>
@@ -6893,4 +7140,1348 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T40"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="13" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="31">
+        <f>'TOTAL RH'!A1</f>
+        <v/>
+      </c>
+      <c r="T1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="T2" s="1" t="n"/>
+    </row>
+    <row r="3" ht="13" customHeight="1">
+      <c r="A3" s="1" t="n"/>
+      <c r="B3" s="1" t="n"/>
+      <c r="C3" s="1" t="n"/>
+      <c r="D3" s="1" t="n"/>
+      <c r="E3" s="1" t="n"/>
+      <c r="F3" s="1" t="n"/>
+      <c r="G3" s="1" t="n"/>
+      <c r="H3" s="1" t="n"/>
+      <c r="I3" s="1" t="n"/>
+      <c r="J3" s="1" t="n"/>
+      <c r="K3" s="1" t="n"/>
+      <c r="L3" s="1" t="n"/>
+      <c r="M3" s="1" t="n"/>
+      <c r="N3" s="1" t="n"/>
+      <c r="O3" s="1" t="n"/>
+      <c r="P3" s="1" t="n"/>
+      <c r="Q3" s="1" t="n"/>
+      <c r="R3" s="1" t="n"/>
+      <c r="S3" s="1" t="n"/>
+      <c r="T3" s="1" t="n"/>
+    </row>
+    <row r="4" ht="13" customHeight="1">
+      <c r="A4" s="1" t="n"/>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>SHORTFALL ALERT</t>
+        </is>
+      </c>
+      <c r="C4" s="53" t="n"/>
+      <c r="D4" s="53" t="n"/>
+      <c r="E4" s="54" t="n"/>
+      <c r="F4" s="1" t="n"/>
+      <c r="G4" s="33" t="inlineStr">
+        <is>
+          <t>COMBINED 40'RH STOCK</t>
+        </is>
+      </c>
+      <c r="H4" s="53" t="n"/>
+      <c r="I4" s="53" t="n"/>
+      <c r="J4" s="54" t="n"/>
+      <c r="K4" s="1" t="n"/>
+      <c r="L4" s="33" t="inlineStr">
+        <is>
+          <t>COMBINED 40'RH BOOKING</t>
+        </is>
+      </c>
+      <c r="M4" s="53" t="n"/>
+      <c r="N4" s="53" t="n"/>
+      <c r="O4" s="54" t="n"/>
+      <c r="P4" s="1" t="n"/>
+      <c r="Q4" s="33" t="inlineStr">
+        <is>
+          <t>COMBINED 40'RH BALANCE</t>
+        </is>
+      </c>
+      <c r="R4" s="53" t="n"/>
+      <c r="S4" s="53" t="n"/>
+      <c r="T4" s="54" t="n"/>
+    </row>
+    <row r="5" ht="13" customHeight="1">
+      <c r="A5" s="1" t="n"/>
+      <c r="B5" s="35">
+        <f>MIN('TOTAL RH'!D12,'TOTAL RH'!J12)</f>
+        <v/>
+      </c>
+      <c r="C5" s="53" t="n"/>
+      <c r="D5" s="53" t="n"/>
+      <c r="E5" s="54" t="n"/>
+      <c r="F5" s="1" t="n"/>
+      <c r="G5" s="36">
+        <f>'TOTAL RH'!O5</f>
+        <v/>
+      </c>
+      <c r="H5" s="53" t="n"/>
+      <c r="I5" s="53" t="n"/>
+      <c r="J5" s="54" t="n"/>
+      <c r="K5" s="1" t="n"/>
+      <c r="L5" s="36">
+        <f>'TOTAL RH'!O10</f>
+        <v/>
+      </c>
+      <c r="M5" s="53" t="n"/>
+      <c r="N5" s="53" t="n"/>
+      <c r="O5" s="54" t="n"/>
+      <c r="P5" s="1" t="n"/>
+      <c r="Q5" s="35">
+        <f>'TOTAL RH'!O15</f>
+        <v/>
+      </c>
+      <c r="R5" s="53" t="n"/>
+      <c r="S5" s="53" t="n"/>
+      <c r="T5" s="54" t="n"/>
+    </row>
+    <row r="6" ht="13" customHeight="1">
+      <c r="A6" s="1" t="n"/>
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>BKK27/LCH27 40'RH, worse balance till 3 OCT</t>
+        </is>
+      </c>
+      <c r="C6" s="53" t="n"/>
+      <c r="D6" s="53" t="n"/>
+      <c r="E6" s="54" t="n"/>
+      <c r="F6" s="1" t="n"/>
+      <c r="G6" s="37" t="inlineStr">
+        <is>
+          <t>BKK27 + LCH27</t>
+        </is>
+      </c>
+      <c r="H6" s="53" t="n"/>
+      <c r="I6" s="53" t="n"/>
+      <c r="J6" s="54" t="n"/>
+      <c r="K6" s="1" t="n"/>
+      <c r="L6" s="37" t="inlineStr">
+        <is>
+          <t>pending + all weeks</t>
+        </is>
+      </c>
+      <c r="M6" s="53" t="n"/>
+      <c r="N6" s="53" t="n"/>
+      <c r="O6" s="54" t="n"/>
+      <c r="P6" s="1" t="n"/>
+      <c r="Q6" s="37" t="inlineStr">
+        <is>
+          <t>till 3 OCT, both depots</t>
+        </is>
+      </c>
+      <c r="R6" s="53" t="n"/>
+      <c r="S6" s="53" t="n"/>
+      <c r="T6" s="54" t="n"/>
+    </row>
+    <row r="7" ht="13" customHeight="1">
+      <c r="A7" s="1" t="n"/>
+      <c r="B7" s="1" t="n"/>
+      <c r="C7" s="1" t="n"/>
+      <c r="D7" s="1" t="n"/>
+      <c r="E7" s="1" t="n"/>
+      <c r="F7" s="1" t="n"/>
+      <c r="G7" s="1" t="n"/>
+      <c r="H7" s="1" t="n"/>
+      <c r="I7" s="1" t="n"/>
+      <c r="J7" s="1" t="n"/>
+      <c r="K7" s="1" t="n"/>
+      <c r="L7" s="1" t="n"/>
+      <c r="M7" s="1" t="n"/>
+      <c r="N7" s="1" t="n"/>
+      <c r="O7" s="1" t="n"/>
+      <c r="P7" s="1" t="n"/>
+      <c r="Q7" s="1" t="n"/>
+      <c r="R7" s="1" t="n"/>
+      <c r="S7" s="1" t="n"/>
+      <c r="T7" s="1" t="n"/>
+    </row>
+    <row r="8" ht="13" customHeight="1">
+      <c r="A8" s="1" t="n"/>
+      <c r="B8" s="38" t="inlineStr">
+        <is>
+          <t>DETAIL BY DEPOT</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n"/>
+      <c r="D8" s="1" t="n"/>
+      <c r="E8" s="1" t="n"/>
+      <c r="F8" s="1" t="n"/>
+      <c r="G8" s="1" t="n"/>
+      <c r="H8" s="1" t="n"/>
+      <c r="I8" s="1" t="n"/>
+      <c r="J8" s="1" t="n"/>
+      <c r="K8" s="1" t="n"/>
+      <c r="L8" s="1" t="n"/>
+      <c r="M8" s="1" t="n"/>
+      <c r="N8" s="1" t="n"/>
+      <c r="O8" s="1" t="n"/>
+      <c r="P8" s="1" t="n"/>
+      <c r="Q8" s="1" t="n"/>
+      <c r="R8" s="1" t="n"/>
+      <c r="S8" s="1" t="n"/>
+      <c r="T8" s="1" t="n"/>
+    </row>
+    <row r="9" ht="13" customHeight="1">
+      <c r="A9" s="1" t="n"/>
+      <c r="B9" s="39">
+        <f>'TOTAL RH'!B2</f>
+        <v/>
+      </c>
+      <c r="C9" s="53" t="n"/>
+      <c r="D9" s="54" t="n"/>
+      <c r="E9" s="1" t="n"/>
+      <c r="F9" s="1" t="n"/>
+      <c r="G9" s="1" t="n"/>
+      <c r="H9" s="1" t="n"/>
+      <c r="I9" s="40">
+        <f>'TOTAL RH'!H2</f>
+        <v/>
+      </c>
+      <c r="J9" s="53" t="n"/>
+      <c r="K9" s="54" t="n"/>
+      <c r="L9" s="1" t="n"/>
+      <c r="M9" s="1" t="n"/>
+      <c r="N9" s="1" t="n"/>
+      <c r="O9" s="1" t="n"/>
+      <c r="P9" s="1" t="n"/>
+      <c r="Q9" s="1" t="n"/>
+      <c r="R9" s="1" t="n"/>
+      <c r="S9" s="1" t="n"/>
+      <c r="T9" s="1" t="n"/>
+    </row>
+    <row r="10" ht="13" customHeight="1">
+      <c r="A10" s="1" t="n"/>
+      <c r="B10" s="34" t="n"/>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="n"/>
+      <c r="F10" s="1" t="n"/>
+      <c r="G10" s="1" t="n"/>
+      <c r="H10" s="1" t="n"/>
+      <c r="I10" s="34" t="n"/>
+      <c r="J10" s="41" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="K10" s="41" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+      <c r="L10" s="1" t="n"/>
+      <c r="M10" s="1" t="n"/>
+      <c r="N10" s="1" t="n"/>
+      <c r="O10" s="1" t="n"/>
+      <c r="P10" s="1" t="n"/>
+      <c r="Q10" s="1" t="n"/>
+      <c r="R10" s="1" t="n"/>
+      <c r="S10" s="1" t="n"/>
+      <c r="T10" s="1" t="n"/>
+    </row>
+    <row r="11" ht="13" customHeight="1">
+      <c r="A11" s="1" t="n"/>
+      <c r="B11" s="42" t="inlineStr">
+        <is>
+          <t>Stock empty in yard</t>
+        </is>
+      </c>
+      <c r="C11" s="43">
+        <f>'TOTAL RH'!C4</f>
+        <v/>
+      </c>
+      <c r="D11" s="43">
+        <f>'TOTAL RH'!D4</f>
+        <v/>
+      </c>
+      <c r="E11" s="1" t="n"/>
+      <c r="F11" s="1" t="n"/>
+      <c r="G11" s="1" t="n"/>
+      <c r="H11" s="1" t="n"/>
+      <c r="I11" s="42" t="inlineStr">
+        <is>
+          <t>Stock empty in yard</t>
+        </is>
+      </c>
+      <c r="J11" s="43">
+        <f>'TOTAL RH'!I4</f>
+        <v/>
+      </c>
+      <c r="K11" s="43">
+        <f>'TOTAL RH'!J4</f>
+        <v/>
+      </c>
+      <c r="L11" s="1" t="n"/>
+      <c r="M11" s="1" t="n"/>
+      <c r="N11" s="1" t="n"/>
+      <c r="O11" s="1" t="n"/>
+      <c r="P11" s="1" t="n"/>
+      <c r="Q11" s="1" t="n"/>
+      <c r="R11" s="1" t="n"/>
+      <c r="S11" s="1" t="n"/>
+      <c r="T11" s="1" t="n"/>
+    </row>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="1" t="n"/>
+      <c r="B12" s="44" t="inlineStr">
+        <is>
+          <t>Booking Pending pick up</t>
+        </is>
+      </c>
+      <c r="C12" s="45">
+        <f>'TOTAL RH'!C5</f>
+        <v/>
+      </c>
+      <c r="D12" s="45">
+        <f>'TOTAL RH'!D5</f>
+        <v/>
+      </c>
+      <c r="E12" s="1" t="n"/>
+      <c r="F12" s="1" t="n"/>
+      <c r="G12" s="1" t="n"/>
+      <c r="H12" s="1" t="n"/>
+      <c r="I12" s="44" t="inlineStr">
+        <is>
+          <t>Booking Pending pick up</t>
+        </is>
+      </c>
+      <c r="J12" s="45">
+        <f>'TOTAL RH'!I5</f>
+        <v/>
+      </c>
+      <c r="K12" s="45">
+        <f>'TOTAL RH'!J5</f>
+        <v/>
+      </c>
+      <c r="L12" s="1" t="n"/>
+      <c r="M12" s="1" t="n"/>
+      <c r="N12" s="1" t="n"/>
+      <c r="O12" s="1" t="n"/>
+      <c r="P12" s="1" t="n"/>
+      <c r="Q12" s="1" t="n"/>
+      <c r="R12" s="1" t="n"/>
+      <c r="S12" s="1" t="n"/>
+      <c r="T12" s="1" t="n"/>
+    </row>
+    <row r="13" ht="13" customHeight="1">
+      <c r="A13" s="1" t="n"/>
+      <c r="B13" s="44" t="inlineStr">
+        <is>
+          <t>Booking on today</t>
+        </is>
+      </c>
+      <c r="C13" s="45">
+        <f>'TOTAL RH'!C6</f>
+        <v/>
+      </c>
+      <c r="D13" s="45">
+        <f>'TOTAL RH'!D6</f>
+        <v/>
+      </c>
+      <c r="E13" s="1" t="n"/>
+      <c r="F13" s="1" t="n"/>
+      <c r="G13" s="1" t="n"/>
+      <c r="H13" s="1" t="n"/>
+      <c r="I13" s="44" t="inlineStr">
+        <is>
+          <t>Booking on today</t>
+        </is>
+      </c>
+      <c r="J13" s="45">
+        <f>'TOTAL RH'!I6</f>
+        <v/>
+      </c>
+      <c r="K13" s="45">
+        <f>'TOTAL RH'!J6</f>
+        <v/>
+      </c>
+      <c r="L13" s="1" t="n"/>
+      <c r="M13" s="1" t="n"/>
+      <c r="N13" s="1" t="n"/>
+      <c r="O13" s="1" t="n"/>
+      <c r="P13" s="1" t="n"/>
+      <c r="Q13" s="1" t="n"/>
+      <c r="R13" s="1" t="n"/>
+      <c r="S13" s="1" t="n"/>
+      <c r="T13" s="1" t="n"/>
+    </row>
+    <row r="14" ht="13" customHeight="1">
+      <c r="A14" s="1" t="n"/>
+      <c r="B14" s="44" t="inlineStr">
+        <is>
+          <t>Booking rest of this week</t>
+        </is>
+      </c>
+      <c r="C14" s="45">
+        <f>'TOTAL RH'!C7</f>
+        <v/>
+      </c>
+      <c r="D14" s="45">
+        <f>'TOTAL RH'!D7</f>
+        <v/>
+      </c>
+      <c r="E14" s="1" t="n"/>
+      <c r="F14" s="1" t="n"/>
+      <c r="G14" s="1" t="n"/>
+      <c r="H14" s="1" t="n"/>
+      <c r="I14" s="44" t="inlineStr">
+        <is>
+          <t>Booking rest of this week</t>
+        </is>
+      </c>
+      <c r="J14" s="45">
+        <f>'TOTAL RH'!I7</f>
+        <v/>
+      </c>
+      <c r="K14" s="45">
+        <f>'TOTAL RH'!J7</f>
+        <v/>
+      </c>
+      <c r="L14" s="1" t="n"/>
+      <c r="M14" s="1" t="n"/>
+      <c r="N14" s="1" t="n"/>
+      <c r="O14" s="1" t="n"/>
+      <c r="P14" s="1" t="n"/>
+      <c r="Q14" s="1" t="n"/>
+      <c r="R14" s="1" t="n"/>
+      <c r="S14" s="1" t="n"/>
+      <c r="T14" s="1" t="n"/>
+    </row>
+    <row r="15" ht="13" customHeight="1">
+      <c r="A15" s="1" t="n"/>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>AV Balance till 19 SEP</t>
+        </is>
+      </c>
+      <c r="C15" s="47">
+        <f>'TOTAL RH'!C8</f>
+        <v/>
+      </c>
+      <c r="D15" s="47">
+        <f>'TOTAL RH'!D8</f>
+        <v/>
+      </c>
+      <c r="E15" s="1" t="n"/>
+      <c r="F15" s="1" t="n"/>
+      <c r="G15" s="1" t="n"/>
+      <c r="H15" s="1" t="n"/>
+      <c r="I15" s="46" t="inlineStr">
+        <is>
+          <t>AV Balance till 19 SEP</t>
+        </is>
+      </c>
+      <c r="J15" s="47">
+        <f>'TOTAL RH'!I8</f>
+        <v/>
+      </c>
+      <c r="K15" s="47">
+        <f>'TOTAL RH'!J8</f>
+        <v/>
+      </c>
+      <c r="L15" s="1" t="n"/>
+      <c r="M15" s="1" t="n"/>
+      <c r="N15" s="1" t="n"/>
+      <c r="O15" s="1" t="n"/>
+      <c r="P15" s="1" t="n"/>
+      <c r="Q15" s="1" t="n"/>
+      <c r="R15" s="1" t="n"/>
+      <c r="S15" s="1" t="n"/>
+      <c r="T15" s="1" t="n"/>
+    </row>
+    <row r="16" ht="13" customHeight="1">
+      <c r="A16" s="1" t="n"/>
+      <c r="B16" s="44" t="inlineStr">
+        <is>
+          <t>Booking 21-26 SEP</t>
+        </is>
+      </c>
+      <c r="C16" s="45">
+        <f>'TOTAL RH'!C9</f>
+        <v/>
+      </c>
+      <c r="D16" s="45">
+        <f>'TOTAL RH'!D9</f>
+        <v/>
+      </c>
+      <c r="E16" s="1" t="n"/>
+      <c r="F16" s="1" t="n"/>
+      <c r="G16" s="1" t="n"/>
+      <c r="H16" s="1" t="n"/>
+      <c r="I16" s="44" t="inlineStr">
+        <is>
+          <t>Booking 21-26 SEP</t>
+        </is>
+      </c>
+      <c r="J16" s="45">
+        <f>'TOTAL RH'!I9</f>
+        <v/>
+      </c>
+      <c r="K16" s="45">
+        <f>'TOTAL RH'!J9</f>
+        <v/>
+      </c>
+      <c r="L16" s="1" t="n"/>
+      <c r="M16" s="1" t="n"/>
+      <c r="N16" s="1" t="n"/>
+      <c r="O16" s="1" t="n"/>
+      <c r="P16" s="1" t="n"/>
+      <c r="Q16" s="1" t="n"/>
+      <c r="R16" s="1" t="n"/>
+      <c r="S16" s="1" t="n"/>
+      <c r="T16" s="1" t="n"/>
+    </row>
+    <row r="17" ht="13" customHeight="1">
+      <c r="A17" s="1" t="n"/>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>AV Balance till 26 SEP</t>
+        </is>
+      </c>
+      <c r="C17" s="47">
+        <f>'TOTAL RH'!C10</f>
+        <v/>
+      </c>
+      <c r="D17" s="55">
+        <f>'TOTAL RH'!D10</f>
+        <v/>
+      </c>
+      <c r="E17" s="1" t="n"/>
+      <c r="F17" s="1" t="n"/>
+      <c r="G17" s="1" t="n"/>
+      <c r="H17" s="1" t="n"/>
+      <c r="I17" s="46" t="inlineStr">
+        <is>
+          <t>AV Balance till 26 SEP</t>
+        </is>
+      </c>
+      <c r="J17" s="47">
+        <f>'TOTAL RH'!I10</f>
+        <v/>
+      </c>
+      <c r="K17" s="47">
+        <f>'TOTAL RH'!J10</f>
+        <v/>
+      </c>
+      <c r="L17" s="1" t="n"/>
+      <c r="M17" s="1" t="n"/>
+      <c r="N17" s="1" t="n"/>
+      <c r="O17" s="1" t="n"/>
+      <c r="P17" s="1" t="n"/>
+      <c r="Q17" s="1" t="n"/>
+      <c r="R17" s="1" t="n"/>
+      <c r="S17" s="1" t="n"/>
+      <c r="T17" s="1" t="n"/>
+    </row>
+    <row r="18" ht="13" customHeight="1">
+      <c r="A18" s="1" t="n"/>
+      <c r="B18" s="44" t="inlineStr">
+        <is>
+          <t>Booking 28 SEP-3 OCT</t>
+        </is>
+      </c>
+      <c r="C18" s="45">
+        <f>'TOTAL RH'!C11</f>
+        <v/>
+      </c>
+      <c r="D18" s="45">
+        <f>'TOTAL RH'!D11</f>
+        <v/>
+      </c>
+      <c r="E18" s="1" t="n"/>
+      <c r="F18" s="1" t="n"/>
+      <c r="G18" s="1" t="n"/>
+      <c r="H18" s="1" t="n"/>
+      <c r="I18" s="44" t="inlineStr">
+        <is>
+          <t>Booking 28 SEP-3 OCT</t>
+        </is>
+      </c>
+      <c r="J18" s="45">
+        <f>'TOTAL RH'!I11</f>
+        <v/>
+      </c>
+      <c r="K18" s="45">
+        <f>'TOTAL RH'!J11</f>
+        <v/>
+      </c>
+      <c r="L18" s="1" t="n"/>
+      <c r="M18" s="1" t="n"/>
+      <c r="N18" s="1" t="n"/>
+      <c r="O18" s="1" t="n"/>
+      <c r="P18" s="1" t="n"/>
+      <c r="Q18" s="1" t="n"/>
+      <c r="R18" s="1" t="n"/>
+      <c r="S18" s="1" t="n"/>
+      <c r="T18" s="1" t="n"/>
+    </row>
+    <row r="19" ht="13" customHeight="1">
+      <c r="A19" s="1" t="n"/>
+      <c r="B19" s="46" t="inlineStr">
+        <is>
+          <t>AV Balance till 3 OCT</t>
+        </is>
+      </c>
+      <c r="C19" s="47">
+        <f>'TOTAL RH'!C12</f>
+        <v/>
+      </c>
+      <c r="D19" s="55">
+        <f>'TOTAL RH'!D12</f>
+        <v/>
+      </c>
+      <c r="E19" s="1" t="n"/>
+      <c r="F19" s="1" t="n"/>
+      <c r="G19" s="1" t="n"/>
+      <c r="H19" s="1" t="n"/>
+      <c r="I19" s="46" t="inlineStr">
+        <is>
+          <t>AV Balance till 3 OCT</t>
+        </is>
+      </c>
+      <c r="J19" s="47">
+        <f>'TOTAL RH'!I12</f>
+        <v/>
+      </c>
+      <c r="K19" s="55">
+        <f>'TOTAL RH'!J12</f>
+        <v/>
+      </c>
+      <c r="L19" s="1" t="n"/>
+      <c r="M19" s="1" t="n"/>
+      <c r="N19" s="1" t="n"/>
+      <c r="O19" s="1" t="n"/>
+      <c r="P19" s="1" t="n"/>
+      <c r="Q19" s="1" t="n"/>
+      <c r="R19" s="1" t="n"/>
+      <c r="S19" s="1" t="n"/>
+      <c r="T19" s="1" t="n"/>
+    </row>
+    <row r="20" ht="13" customHeight="1">
+      <c r="A20" s="1" t="n"/>
+      <c r="B20" s="1" t="n"/>
+      <c r="C20" s="1" t="n"/>
+      <c r="D20" s="1" t="n"/>
+      <c r="E20" s="1" t="n"/>
+      <c r="F20" s="1" t="n"/>
+      <c r="G20" s="1" t="n"/>
+      <c r="H20" s="1" t="n"/>
+      <c r="I20" s="1" t="n"/>
+      <c r="J20" s="1" t="n"/>
+      <c r="K20" s="1" t="n"/>
+      <c r="L20" s="1" t="n"/>
+      <c r="M20" s="1" t="n"/>
+      <c r="N20" s="1" t="n"/>
+      <c r="O20" s="1" t="n"/>
+      <c r="P20" s="1" t="n"/>
+      <c r="Q20" s="1" t="n"/>
+      <c r="R20" s="1" t="n"/>
+      <c r="S20" s="1" t="n"/>
+      <c r="T20" s="1" t="n"/>
+    </row>
+    <row r="21" ht="13" customHeight="1">
+      <c r="A21" s="1" t="n"/>
+      <c r="B21" s="1" t="n"/>
+      <c r="C21" s="1" t="n"/>
+      <c r="D21" s="1" t="n"/>
+      <c r="E21" s="1" t="n"/>
+      <c r="F21" s="1" t="n"/>
+      <c r="G21" s="1" t="n"/>
+      <c r="H21" s="1" t="n"/>
+      <c r="I21" s="1" t="n"/>
+      <c r="J21" s="1" t="n"/>
+      <c r="K21" s="1" t="n"/>
+      <c r="L21" s="1" t="n"/>
+      <c r="M21" s="1" t="n"/>
+      <c r="N21" s="1" t="n"/>
+      <c r="O21" s="1" t="n"/>
+      <c r="P21" s="1" t="n"/>
+      <c r="Q21" s="1" t="n"/>
+      <c r="R21" s="1" t="n"/>
+      <c r="S21" s="1" t="n"/>
+      <c r="T21" s="1" t="n"/>
+    </row>
+    <row r="22" ht="13" customHeight="1">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t>REMARKS  (AV = move code IED/IEP/IER, DMG = move code OER)</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="n"/>
+      <c r="D22" s="1" t="n"/>
+      <c r="E22" s="1" t="n"/>
+      <c r="F22" s="1" t="n"/>
+      <c r="G22" s="1" t="n"/>
+      <c r="H22" s="1" t="n"/>
+      <c r="I22" s="1" t="n"/>
+      <c r="J22" s="1" t="n"/>
+      <c r="K22" s="1" t="n"/>
+      <c r="L22" s="1" t="n"/>
+      <c r="M22" s="1" t="n"/>
+      <c r="N22" s="1" t="n"/>
+      <c r="O22" s="1" t="n"/>
+      <c r="P22" s="1" t="n"/>
+      <c r="Q22" s="1" t="n"/>
+      <c r="R22" s="1" t="n"/>
+      <c r="S22" s="1" t="n"/>
+      <c r="T22" s="1" t="n"/>
+    </row>
+    <row r="23" ht="13" customHeight="1">
+      <c r="A23" s="1" t="n"/>
+      <c r="B23" s="39">
+        <f>'TOTAL RH'!B2</f>
+        <v/>
+      </c>
+      <c r="C23" s="53" t="n"/>
+      <c r="D23" s="54" t="n"/>
+      <c r="E23" s="1" t="n"/>
+      <c r="F23" s="1" t="n"/>
+      <c r="G23" s="1" t="n"/>
+      <c r="H23" s="1" t="n"/>
+      <c r="I23" s="40">
+        <f>'TOTAL RH'!H2</f>
+        <v/>
+      </c>
+      <c r="J23" s="53" t="n"/>
+      <c r="K23" s="54" t="n"/>
+      <c r="L23" s="1" t="n"/>
+      <c r="M23" s="1" t="n"/>
+      <c r="N23" s="1" t="n"/>
+      <c r="O23" s="1" t="n"/>
+      <c r="P23" s="1" t="n"/>
+      <c r="Q23" s="1" t="n"/>
+      <c r="R23" s="1" t="n"/>
+      <c r="S23" s="1" t="n"/>
+      <c r="T23" s="1" t="n"/>
+    </row>
+    <row r="24" ht="13" customHeight="1">
+      <c r="A24" s="1" t="n"/>
+      <c r="B24" s="34" t="n"/>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="D24" s="41" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="n"/>
+      <c r="F24" s="1" t="n"/>
+      <c r="G24" s="1" t="n"/>
+      <c r="H24" s="1" t="n"/>
+      <c r="I24" s="34" t="n"/>
+      <c r="J24" s="41" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
+      <c r="K24" s="41" t="inlineStr">
+        <is>
+          <t>40'RH</t>
+        </is>
+      </c>
+      <c r="L24" s="1" t="n"/>
+      <c r="M24" s="1" t="n"/>
+      <c r="N24" s="1" t="n"/>
+      <c r="O24" s="1" t="n"/>
+      <c r="P24" s="1" t="n"/>
+      <c r="Q24" s="1" t="n"/>
+      <c r="R24" s="1" t="n"/>
+      <c r="S24" s="1" t="n"/>
+      <c r="T24" s="1" t="n"/>
+    </row>
+    <row r="25" ht="13" customHeight="1">
+      <c r="A25" s="1" t="n"/>
+      <c r="B25" s="34" t="inlineStr">
+        <is>
+          <t>AV</t>
+        </is>
+      </c>
+      <c r="C25" s="45">
+        <f>'TOTAL RH'!C16</f>
+        <v/>
+      </c>
+      <c r="D25" s="45">
+        <f>'TOTAL RH'!D16</f>
+        <v/>
+      </c>
+      <c r="E25" s="1" t="n"/>
+      <c r="F25" s="1" t="n"/>
+      <c r="G25" s="1" t="n"/>
+      <c r="H25" s="1" t="n"/>
+      <c r="I25" s="34" t="inlineStr">
+        <is>
+          <t>AV</t>
+        </is>
+      </c>
+      <c r="J25" s="45">
+        <f>'TOTAL RH'!I16</f>
+        <v/>
+      </c>
+      <c r="K25" s="45">
+        <f>'TOTAL RH'!J16</f>
+        <v/>
+      </c>
+      <c r="L25" s="1" t="n"/>
+      <c r="M25" s="1" t="n"/>
+      <c r="N25" s="1" t="n"/>
+      <c r="O25" s="1" t="n"/>
+      <c r="P25" s="1" t="n"/>
+      <c r="Q25" s="1" t="n"/>
+      <c r="R25" s="1" t="n"/>
+      <c r="S25" s="1" t="n"/>
+      <c r="T25" s="1" t="n"/>
+    </row>
+    <row r="26" ht="13" customHeight="1">
+      <c r="A26" s="1" t="n"/>
+      <c r="B26" s="34" t="inlineStr">
+        <is>
+          <t>DMG</t>
+        </is>
+      </c>
+      <c r="C26" s="45">
+        <f>'TOTAL RH'!C17</f>
+        <v/>
+      </c>
+      <c r="D26" s="45">
+        <f>'TOTAL RH'!D17</f>
+        <v/>
+      </c>
+      <c r="E26" s="1" t="n"/>
+      <c r="F26" s="1" t="n"/>
+      <c r="G26" s="1" t="n"/>
+      <c r="H26" s="1" t="n"/>
+      <c r="I26" s="34" t="inlineStr">
+        <is>
+          <t>DMG</t>
+        </is>
+      </c>
+      <c r="J26" s="45">
+        <f>'TOTAL RH'!I17</f>
+        <v/>
+      </c>
+      <c r="K26" s="45">
+        <f>'TOTAL RH'!J17</f>
+        <v/>
+      </c>
+      <c r="L26" s="1" t="n"/>
+      <c r="M26" s="1" t="n"/>
+      <c r="N26" s="1" t="n"/>
+      <c r="O26" s="1" t="n"/>
+      <c r="P26" s="1" t="n"/>
+      <c r="Q26" s="1" t="n"/>
+      <c r="R26" s="1" t="n"/>
+      <c r="S26" s="1" t="n"/>
+      <c r="T26" s="1" t="n"/>
+    </row>
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="1" t="n"/>
+      <c r="B27" s="1" t="n"/>
+      <c r="C27" s="1" t="n"/>
+      <c r="D27" s="1" t="n"/>
+      <c r="E27" s="1" t="n"/>
+      <c r="F27" s="1" t="n"/>
+      <c r="G27" s="1" t="n"/>
+      <c r="H27" s="1" t="n"/>
+      <c r="I27" s="1" t="n"/>
+      <c r="J27" s="1" t="n"/>
+      <c r="K27" s="1" t="n"/>
+      <c r="L27" s="1" t="n"/>
+      <c r="M27" s="1" t="n"/>
+      <c r="N27" s="1" t="n"/>
+      <c r="O27" s="1" t="n"/>
+      <c r="P27" s="1" t="n"/>
+      <c r="Q27" s="1" t="n"/>
+      <c r="R27" s="1" t="n"/>
+      <c r="S27" s="1" t="n"/>
+      <c r="T27" s="1" t="n"/>
+    </row>
+    <row r="28" ht="13" customHeight="1">
+      <c r="A28" s="1" t="n"/>
+      <c r="B28" s="1" t="n"/>
+      <c r="C28" s="1" t="n"/>
+      <c r="D28" s="1" t="n"/>
+      <c r="E28" s="1" t="n"/>
+      <c r="F28" s="1" t="n"/>
+      <c r="G28" s="1" t="n"/>
+      <c r="H28" s="1" t="n"/>
+      <c r="I28" s="1" t="n"/>
+      <c r="J28" s="1" t="n"/>
+      <c r="K28" s="1" t="n"/>
+      <c r="L28" s="1" t="n"/>
+      <c r="M28" s="1" t="n"/>
+      <c r="N28" s="1" t="n"/>
+      <c r="O28" s="1" t="n"/>
+      <c r="P28" s="1" t="n"/>
+      <c r="Q28" s="1" t="n"/>
+      <c r="R28" s="1" t="n"/>
+      <c r="S28" s="1" t="n"/>
+      <c r="T28" s="1" t="n"/>
+    </row>
+    <row r="29" ht="13" customHeight="1">
+      <c r="A29" s="1" t="n"/>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>RF SEASONAL — build year</t>
+        </is>
+      </c>
+      <c r="C29" s="1" t="n"/>
+      <c r="D29" s="1" t="n"/>
+      <c r="E29" s="1" t="n"/>
+      <c r="F29" s="1" t="n"/>
+      <c r="G29" s="1" t="n"/>
+      <c r="H29" s="1" t="n"/>
+      <c r="I29" s="1" t="n"/>
+      <c r="J29" s="1" t="n"/>
+      <c r="K29" s="1" t="n"/>
+      <c r="L29" s="1" t="n"/>
+      <c r="M29" s="1" t="n"/>
+      <c r="N29" s="1" t="n"/>
+      <c r="O29" s="1" t="n"/>
+      <c r="P29" s="1" t="n"/>
+      <c r="Q29" s="1" t="n"/>
+      <c r="R29" s="1" t="n"/>
+      <c r="S29" s="1" t="n"/>
+      <c r="T29" s="1" t="n"/>
+    </row>
+    <row r="30" ht="13" customHeight="1">
+      <c r="A30" s="1" t="n"/>
+      <c r="B30" s="33" t="inlineStr">
+        <is>
+          <t>BKK27 2020-26 BUILT</t>
+        </is>
+      </c>
+      <c r="C30" s="53" t="n"/>
+      <c r="D30" s="53" t="n"/>
+      <c r="E30" s="54" t="n"/>
+      <c r="F30" s="1" t="n"/>
+      <c r="G30" s="33" t="inlineStr">
+        <is>
+          <t>LCH27 2020-26 BUILT</t>
+        </is>
+      </c>
+      <c r="H30" s="53" t="n"/>
+      <c r="I30" s="53" t="n"/>
+      <c r="J30" s="54" t="n"/>
+      <c r="K30" s="1" t="n"/>
+      <c r="L30" s="33" t="inlineStr">
+        <is>
+          <t>PEAK BUILD YEAR</t>
+        </is>
+      </c>
+      <c r="M30" s="53" t="n"/>
+      <c r="N30" s="53" t="n"/>
+      <c r="O30" s="54" t="n"/>
+      <c r="P30" s="1" t="n"/>
+      <c r="Q30" s="1" t="n"/>
+      <c r="R30" s="1" t="n"/>
+      <c r="S30" s="1" t="n"/>
+      <c r="T30" s="1" t="n"/>
+    </row>
+    <row r="31" ht="13" customHeight="1">
+      <c r="A31" s="1" t="n"/>
+      <c r="B31" s="48">
+        <f>SUM('TOTAL RH'!D36:D42)+SUM('TOTAL RH'!F36:F42)+SUM('TOTAL RH'!H36:H42)</f>
+        <v/>
+      </c>
+      <c r="C31" s="53" t="n"/>
+      <c r="D31" s="53" t="n"/>
+      <c r="E31" s="54" t="n"/>
+      <c r="F31" s="1" t="n"/>
+      <c r="G31" s="49">
+        <f>SUM('TOTAL RH'!L36:L42)+SUM('TOTAL RH'!N36:N42)+SUM('TOTAL RH'!P36:P42)</f>
+        <v/>
+      </c>
+      <c r="H31" s="53" t="n"/>
+      <c r="I31" s="53" t="n"/>
+      <c r="J31" s="54" t="n"/>
+      <c r="K31" s="1" t="n"/>
+      <c r="L31" s="36">
+        <f>"2021 / 2019"</f>
+        <v/>
+      </c>
+      <c r="M31" s="53" t="n"/>
+      <c r="N31" s="53" t="n"/>
+      <c r="O31" s="54" t="n"/>
+      <c r="P31" s="1" t="n"/>
+      <c r="Q31" s="1" t="n"/>
+      <c r="R31" s="1" t="n"/>
+      <c r="S31" s="1" t="n"/>
+      <c r="T31" s="1" t="n"/>
+    </row>
+    <row r="32" ht="13" customHeight="1">
+      <c r="A32" s="1" t="n"/>
+      <c r="B32" s="37" t="inlineStr">
+        <is>
+          <t>of 40'RH on hand</t>
+        </is>
+      </c>
+      <c r="C32" s="53" t="n"/>
+      <c r="D32" s="53" t="n"/>
+      <c r="E32" s="54" t="n"/>
+      <c r="F32" s="1" t="n"/>
+      <c r="G32" s="37" t="inlineStr">
+        <is>
+          <t>of 40'RH on hand</t>
+        </is>
+      </c>
+      <c r="H32" s="53" t="n"/>
+      <c r="I32" s="53" t="n"/>
+      <c r="J32" s="54" t="n"/>
+      <c r="K32" s="1" t="n"/>
+      <c r="L32" s="37" t="inlineStr">
+        <is>
+          <t>19 units across both depots</t>
+        </is>
+      </c>
+      <c r="M32" s="53" t="n"/>
+      <c r="N32" s="53" t="n"/>
+      <c r="O32" s="54" t="n"/>
+      <c r="P32" s="1" t="n"/>
+      <c r="Q32" s="1" t="n"/>
+      <c r="R32" s="1" t="n"/>
+      <c r="S32" s="1" t="n"/>
+      <c r="T32" s="1" t="n"/>
+    </row>
+    <row r="33" ht="13" customHeight="1">
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="1" t="n"/>
+      <c r="C33" s="1" t="n"/>
+      <c r="D33" s="1" t="n"/>
+      <c r="E33" s="1" t="n"/>
+      <c r="F33" s="1" t="n"/>
+      <c r="G33" s="1" t="n"/>
+      <c r="H33" s="1" t="n"/>
+      <c r="I33" s="1" t="n"/>
+      <c r="J33" s="1" t="n"/>
+      <c r="K33" s="1" t="n"/>
+      <c r="L33" s="1" t="n"/>
+      <c r="M33" s="1" t="n"/>
+      <c r="N33" s="1" t="n"/>
+      <c r="O33" s="1" t="n"/>
+      <c r="P33" s="1" t="n"/>
+      <c r="Q33" s="1" t="n"/>
+      <c r="R33" s="1" t="n"/>
+      <c r="S33" s="1" t="n"/>
+      <c r="T33" s="1" t="n"/>
+    </row>
+    <row r="34" ht="13" customHeight="1">
+      <c r="A34" s="1" t="n"/>
+      <c r="B34" s="39" t="inlineStr">
+        <is>
+          <t>BKK27 current mix</t>
+        </is>
+      </c>
+      <c r="C34" s="53" t="n"/>
+      <c r="D34" s="54" t="n"/>
+      <c r="E34" s="1" t="n"/>
+      <c r="F34" s="1" t="n"/>
+      <c r="G34" s="1" t="n"/>
+      <c r="H34" s="1" t="n"/>
+      <c r="I34" s="40" t="inlineStr">
+        <is>
+          <t>LCH27 current mix</t>
+        </is>
+      </c>
+      <c r="J34" s="53" t="n"/>
+      <c r="K34" s="54" t="n"/>
+      <c r="L34" s="1" t="n"/>
+      <c r="M34" s="1" t="n"/>
+      <c r="N34" s="1" t="n"/>
+      <c r="O34" s="1" t="n"/>
+      <c r="P34" s="1" t="n"/>
+      <c r="Q34" s="1" t="n"/>
+      <c r="R34" s="1" t="n"/>
+      <c r="S34" s="1" t="n"/>
+      <c r="T34" s="1" t="n"/>
+    </row>
+    <row r="35" ht="13" customHeight="1">
+      <c r="A35" s="1" t="n"/>
+      <c r="B35" s="34" t="n"/>
+      <c r="C35" s="41" t="inlineStr">
+        <is>
+          <t>22RE</t>
+        </is>
+      </c>
+      <c r="D35" s="41" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="n"/>
+      <c r="F35" s="1" t="n"/>
+      <c r="G35" s="1" t="n"/>
+      <c r="H35" s="1" t="n"/>
+      <c r="I35" s="34" t="n"/>
+      <c r="J35" s="41" t="inlineStr">
+        <is>
+          <t>22RE</t>
+        </is>
+      </c>
+      <c r="K35" s="41" t="inlineStr">
+        <is>
+          <t>45RE</t>
+        </is>
+      </c>
+      <c r="L35" s="1" t="n"/>
+      <c r="M35" s="1" t="n"/>
+      <c r="N35" s="1" t="n"/>
+      <c r="O35" s="1" t="n"/>
+      <c r="P35" s="1" t="n"/>
+      <c r="Q35" s="1" t="n"/>
+      <c r="R35" s="1" t="n"/>
+      <c r="S35" s="1" t="n"/>
+      <c r="T35" s="1" t="n"/>
+    </row>
+    <row r="36" ht="13" customHeight="1">
+      <c r="A36" s="1" t="n"/>
+      <c r="B36" s="34" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="C36" s="45">
+        <f>'TOTAL RH'!C53</f>
+        <v/>
+      </c>
+      <c r="D36" s="45">
+        <f>'TOTAL RH'!D53</f>
+        <v/>
+      </c>
+      <c r="E36" s="1" t="n"/>
+      <c r="F36" s="1" t="n"/>
+      <c r="G36" s="1" t="n"/>
+      <c r="H36" s="1" t="n"/>
+      <c r="I36" s="34" t="inlineStr">
+        <is>
+          <t>CARRIER</t>
+        </is>
+      </c>
+      <c r="J36" s="45">
+        <f>'TOTAL RH'!K53</f>
+        <v/>
+      </c>
+      <c r="K36" s="45">
+        <f>'TOTAL RH'!L53</f>
+        <v/>
+      </c>
+      <c r="L36" s="1" t="n"/>
+      <c r="M36" s="1" t="n"/>
+      <c r="N36" s="1" t="n"/>
+      <c r="O36" s="1" t="n"/>
+      <c r="P36" s="1" t="n"/>
+      <c r="Q36" s="1" t="n"/>
+      <c r="R36" s="1" t="n"/>
+      <c r="S36" s="1" t="n"/>
+      <c r="T36" s="1" t="n"/>
+    </row>
+    <row r="37" ht="13" customHeight="1">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="34" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="C37" s="45">
+        <f>'TOTAL RH'!E53</f>
+        <v/>
+      </c>
+      <c r="D37" s="45">
+        <f>'TOTAL RH'!F53</f>
+        <v/>
+      </c>
+      <c r="E37" s="1" t="n"/>
+      <c r="F37" s="1" t="n"/>
+      <c r="G37" s="1" t="n"/>
+      <c r="H37" s="1" t="n"/>
+      <c r="I37" s="34" t="inlineStr">
+        <is>
+          <t>DAIKIN</t>
+        </is>
+      </c>
+      <c r="J37" s="45">
+        <f>'TOTAL RH'!M53</f>
+        <v/>
+      </c>
+      <c r="K37" s="45">
+        <f>'TOTAL RH'!N53</f>
+        <v/>
+      </c>
+      <c r="L37" s="1" t="n"/>
+      <c r="M37" s="1" t="n"/>
+      <c r="N37" s="1" t="n"/>
+      <c r="O37" s="1" t="n"/>
+      <c r="P37" s="1" t="n"/>
+      <c r="Q37" s="1" t="n"/>
+      <c r="R37" s="1" t="n"/>
+      <c r="S37" s="1" t="n"/>
+      <c r="T37" s="1" t="n"/>
+    </row>
+    <row r="38" ht="13" customHeight="1">
+      <c r="A38" s="1" t="n"/>
+      <c r="B38" s="34" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
+      <c r="C38" s="45">
+        <f>'TOTAL RH'!G53</f>
+        <v/>
+      </c>
+      <c r="D38" s="45">
+        <f>'TOTAL RH'!H53</f>
+        <v/>
+      </c>
+      <c r="E38" s="1" t="n"/>
+      <c r="F38" s="1" t="n"/>
+      <c r="G38" s="1" t="n"/>
+      <c r="H38" s="1" t="n"/>
+      <c r="I38" s="34" t="inlineStr">
+        <is>
+          <t>THERMO KING</t>
+        </is>
+      </c>
+      <c r="J38" s="45">
+        <f>'TOTAL RH'!O53</f>
+        <v/>
+      </c>
+      <c r="K38" s="45">
+        <f>'TOTAL RH'!P53</f>
+        <v/>
+      </c>
+      <c r="L38" s="1" t="n"/>
+      <c r="M38" s="1" t="n"/>
+      <c r="N38" s="1" t="n"/>
+      <c r="O38" s="1" t="n"/>
+      <c r="P38" s="1" t="n"/>
+      <c r="Q38" s="1" t="n"/>
+      <c r="R38" s="1" t="n"/>
+      <c r="S38" s="1" t="n"/>
+      <c r="T38" s="1" t="n"/>
+    </row>
+    <row r="39" ht="13" customHeight="1">
+      <c r="A39" s="1" t="n"/>
+      <c r="B39" s="1" t="n"/>
+      <c r="C39" s="1" t="n"/>
+      <c r="D39" s="1" t="n"/>
+      <c r="E39" s="1" t="n"/>
+      <c r="F39" s="1" t="n"/>
+      <c r="G39" s="1" t="n"/>
+      <c r="H39" s="1" t="n"/>
+      <c r="I39" s="1" t="n"/>
+      <c r="J39" s="1" t="n"/>
+      <c r="K39" s="1" t="n"/>
+      <c r="L39" s="1" t="n"/>
+      <c r="M39" s="1" t="n"/>
+      <c r="N39" s="1" t="n"/>
+      <c r="O39" s="1" t="n"/>
+      <c r="P39" s="1" t="n"/>
+      <c r="Q39" s="1" t="n"/>
+      <c r="R39" s="1" t="n"/>
+      <c r="S39" s="1" t="n"/>
+      <c r="T39" s="1" t="n"/>
+    </row>
+    <row r="40" ht="13" customHeight="1">
+      <c r="A40" s="1" t="n"/>
+      <c r="B40" s="50" t="inlineStr">
+        <is>
+          <t>Full 2010-2026 Year x Brand x Size breakdown is on the TOTAL RH sheet.</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="n"/>
+      <c r="D40" s="1" t="n"/>
+      <c r="E40" s="1" t="n"/>
+      <c r="F40" s="1" t="n"/>
+      <c r="G40" s="1" t="n"/>
+      <c r="H40" s="1" t="n"/>
+      <c r="I40" s="1" t="n"/>
+      <c r="J40" s="1" t="n"/>
+      <c r="K40" s="1" t="n"/>
+      <c r="L40" s="1" t="n"/>
+      <c r="M40" s="1" t="n"/>
+      <c r="N40" s="1" t="n"/>
+      <c r="O40" s="1" t="n"/>
+      <c r="P40" s="1" t="n"/>
+      <c r="Q40" s="1" t="n"/>
+      <c r="R40" s="1" t="n"/>
+      <c r="S40" s="1" t="n"/>
+      <c r="T40" s="1" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="28">
+    <mergeCell ref="L31:O31"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="I23:K23"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="L32:O32"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="I34:K34"/>
+    <mergeCell ref="Q5:T5"/>
+    <mergeCell ref="L5:O5"/>
+    <mergeCell ref="G6:J6"/>
+    <mergeCell ref="Q4:T4"/>
+    <mergeCell ref="L30:O30"/>
+    <mergeCell ref="B1:S2"/>
+    <mergeCell ref="L4:O4"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="Q6:T6"/>
+    <mergeCell ref="G5:J5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tighten Dashboard sheet layout
- Un-merge the KPI stat cards (label/value/desc were merged across
  4 columns each - simplify to single cells with natural overflow,
  matching a hand-edit the user made after the first version).
- Narrow the card widths (4 cols -> 3) and add explicit 2.5-wide
  spacer columns everywhere else on the sheet instead of leaving
  them at Excel's default width, shrinking the sheet from ~20 used
  columns to 16.
- Shave one gap column between the BKK27 and LCH27 blocks in the
  Detail-by-depot / Remarks tables (LCH27 now starts at column H).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Stock_Daily_Reefer_9-17.xlsx
+++ b/Stock_Daily_Reefer_9-17.xlsx
@@ -7148,17 +7148,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T40"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="3" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="2.5" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="2.5" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">
@@ -7167,11 +7168,9 @@
         <f>'TOTAL RH'!A1</f>
         <v/>
       </c>
-      <c r="T1" s="1" t="n"/>
     </row>
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="1" t="n"/>
-      <c r="T2" s="1" t="n"/>
     </row>
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="1" t="n"/>
@@ -7190,10 +7189,6 @@
       <c r="N3" s="1" t="n"/>
       <c r="O3" s="1" t="n"/>
       <c r="P3" s="1" t="n"/>
-      <c r="Q3" s="1" t="n"/>
-      <c r="R3" s="1" t="n"/>
-      <c r="S3" s="1" t="n"/>
-      <c r="T3" s="1" t="n"/>
     </row>
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="1" t="n"/>
@@ -7202,36 +7197,32 @@
           <t>SHORTFALL ALERT</t>
         </is>
       </c>
-      <c r="C4" s="53" t="n"/>
-      <c r="D4" s="53" t="n"/>
-      <c r="E4" s="54" t="n"/>
-      <c r="F4" s="1" t="n"/>
-      <c r="G4" s="33" t="inlineStr">
+      <c r="C4" s="34" t="n"/>
+      <c r="D4" s="34" t="n"/>
+      <c r="E4" s="1" t="n"/>
+      <c r="F4" s="33" t="inlineStr">
         <is>
           <t>COMBINED 40'RH STOCK</t>
         </is>
       </c>
-      <c r="H4" s="53" t="n"/>
-      <c r="I4" s="53" t="n"/>
-      <c r="J4" s="54" t="n"/>
-      <c r="K4" s="1" t="n"/>
-      <c r="L4" s="33" t="inlineStr">
+      <c r="G4" s="34" t="n"/>
+      <c r="H4" s="34" t="n"/>
+      <c r="I4" s="1" t="n"/>
+      <c r="J4" s="33" t="inlineStr">
         <is>
           <t>COMBINED 40'RH BOOKING</t>
         </is>
       </c>
-      <c r="M4" s="53" t="n"/>
-      <c r="N4" s="53" t="n"/>
-      <c r="O4" s="54" t="n"/>
-      <c r="P4" s="1" t="n"/>
-      <c r="Q4" s="33" t="inlineStr">
+      <c r="K4" s="34" t="n"/>
+      <c r="L4" s="34" t="n"/>
+      <c r="M4" s="1" t="n"/>
+      <c r="N4" s="33" t="inlineStr">
         <is>
           <t>COMBINED 40'RH BALANCE</t>
         </is>
       </c>
-      <c r="R4" s="53" t="n"/>
-      <c r="S4" s="53" t="n"/>
-      <c r="T4" s="54" t="n"/>
+      <c r="O4" s="34" t="n"/>
+      <c r="P4" s="34" t="n"/>
     </row>
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="1" t="n"/>
@@ -7239,33 +7230,29 @@
         <f>MIN('TOTAL RH'!D12,'TOTAL RH'!J12)</f>
         <v/>
       </c>
-      <c r="C5" s="53" t="n"/>
-      <c r="D5" s="53" t="n"/>
-      <c r="E5" s="54" t="n"/>
-      <c r="F5" s="1" t="n"/>
-      <c r="G5" s="36">
+      <c r="C5" s="34" t="n"/>
+      <c r="D5" s="34" t="n"/>
+      <c r="E5" s="1" t="n"/>
+      <c r="F5" s="36">
         <f>'TOTAL RH'!O5</f>
         <v/>
       </c>
-      <c r="H5" s="53" t="n"/>
-      <c r="I5" s="53" t="n"/>
-      <c r="J5" s="54" t="n"/>
-      <c r="K5" s="1" t="n"/>
-      <c r="L5" s="36">
+      <c r="G5" s="34" t="n"/>
+      <c r="H5" s="34" t="n"/>
+      <c r="I5" s="1" t="n"/>
+      <c r="J5" s="36">
         <f>'TOTAL RH'!O10</f>
         <v/>
       </c>
-      <c r="M5" s="53" t="n"/>
-      <c r="N5" s="53" t="n"/>
-      <c r="O5" s="54" t="n"/>
-      <c r="P5" s="1" t="n"/>
-      <c r="Q5" s="35">
+      <c r="K5" s="34" t="n"/>
+      <c r="L5" s="34" t="n"/>
+      <c r="M5" s="1" t="n"/>
+      <c r="N5" s="35">
         <f>'TOTAL RH'!O15</f>
         <v/>
       </c>
-      <c r="R5" s="53" t="n"/>
-      <c r="S5" s="53" t="n"/>
-      <c r="T5" s="54" t="n"/>
+      <c r="O5" s="34" t="n"/>
+      <c r="P5" s="34" t="n"/>
     </row>
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="1" t="n"/>
@@ -7274,36 +7261,32 @@
           <t>BKK27/LCH27 40'RH, worse balance till 3 OCT</t>
         </is>
       </c>
-      <c r="C6" s="53" t="n"/>
-      <c r="D6" s="53" t="n"/>
-      <c r="E6" s="54" t="n"/>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="37" t="inlineStr">
+      <c r="C6" s="34" t="n"/>
+      <c r="D6" s="34" t="n"/>
+      <c r="E6" s="1" t="n"/>
+      <c r="F6" s="37" t="inlineStr">
         <is>
           <t>BKK27 + LCH27</t>
         </is>
       </c>
-      <c r="H6" s="53" t="n"/>
-      <c r="I6" s="53" t="n"/>
-      <c r="J6" s="54" t="n"/>
-      <c r="K6" s="1" t="n"/>
-      <c r="L6" s="37" t="inlineStr">
+      <c r="G6" s="34" t="n"/>
+      <c r="H6" s="34" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="37" t="inlineStr">
         <is>
           <t>pending + all weeks</t>
         </is>
       </c>
-      <c r="M6" s="53" t="n"/>
-      <c r="N6" s="53" t="n"/>
-      <c r="O6" s="54" t="n"/>
-      <c r="P6" s="1" t="n"/>
-      <c r="Q6" s="37" t="inlineStr">
+      <c r="K6" s="34" t="n"/>
+      <c r="L6" s="34" t="n"/>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="37" t="inlineStr">
         <is>
           <t>till 3 OCT, both depots</t>
         </is>
       </c>
-      <c r="R6" s="53" t="n"/>
-      <c r="S6" s="53" t="n"/>
-      <c r="T6" s="54" t="n"/>
+      <c r="O6" s="34" t="n"/>
+      <c r="P6" s="34" t="n"/>
     </row>
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="1" t="n"/>
@@ -7322,10 +7305,6 @@
       <c r="N7" s="1" t="n"/>
       <c r="O7" s="1" t="n"/>
       <c r="P7" s="1" t="n"/>
-      <c r="Q7" s="1" t="n"/>
-      <c r="R7" s="1" t="n"/>
-      <c r="S7" s="1" t="n"/>
-      <c r="T7" s="1" t="n"/>
     </row>
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="1" t="n"/>
@@ -7348,10 +7327,6 @@
       <c r="N8" s="1" t="n"/>
       <c r="O8" s="1" t="n"/>
       <c r="P8" s="1" t="n"/>
-      <c r="Q8" s="1" t="n"/>
-      <c r="R8" s="1" t="n"/>
-      <c r="S8" s="1" t="n"/>
-      <c r="T8" s="1" t="n"/>
     </row>
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="1" t="n"/>
@@ -7364,22 +7339,18 @@
       <c r="E9" s="1" t="n"/>
       <c r="F9" s="1" t="n"/>
       <c r="G9" s="1" t="n"/>
-      <c r="H9" s="1" t="n"/>
-      <c r="I9" s="40">
+      <c r="H9" s="40">
         <f>'TOTAL RH'!H2</f>
         <v/>
       </c>
-      <c r="J9" s="53" t="n"/>
-      <c r="K9" s="54" t="n"/>
+      <c r="I9" s="53" t="n"/>
+      <c r="J9" s="54" t="n"/>
+      <c r="K9" s="1" t="n"/>
       <c r="L9" s="1" t="n"/>
       <c r="M9" s="1" t="n"/>
       <c r="N9" s="1" t="n"/>
       <c r="O9" s="1" t="n"/>
       <c r="P9" s="1" t="n"/>
-      <c r="Q9" s="1" t="n"/>
-      <c r="R9" s="1" t="n"/>
-      <c r="S9" s="1" t="n"/>
-      <c r="T9" s="1" t="n"/>
     </row>
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="1" t="n"/>
@@ -7397,27 +7368,23 @@
       <c r="E10" s="1" t="n"/>
       <c r="F10" s="1" t="n"/>
       <c r="G10" s="1" t="n"/>
-      <c r="H10" s="1" t="n"/>
-      <c r="I10" s="34" t="n"/>
+      <c r="H10" s="34" t="n"/>
+      <c r="I10" s="41" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
       <c r="J10" s="41" t="inlineStr">
         <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="K10" s="41" t="inlineStr">
-        <is>
           <t>40'RH</t>
         </is>
       </c>
+      <c r="K10" s="1" t="n"/>
       <c r="L10" s="1" t="n"/>
       <c r="M10" s="1" t="n"/>
       <c r="N10" s="1" t="n"/>
       <c r="O10" s="1" t="n"/>
       <c r="P10" s="1" t="n"/>
-      <c r="Q10" s="1" t="n"/>
-      <c r="R10" s="1" t="n"/>
-      <c r="S10" s="1" t="n"/>
-      <c r="T10" s="1" t="n"/>
     </row>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="1" t="n"/>
@@ -7437,29 +7404,25 @@
       <c r="E11" s="1" t="n"/>
       <c r="F11" s="1" t="n"/>
       <c r="G11" s="1" t="n"/>
-      <c r="H11" s="1" t="n"/>
-      <c r="I11" s="42" t="inlineStr">
+      <c r="H11" s="42" t="inlineStr">
         <is>
           <t>Stock empty in yard</t>
         </is>
       </c>
+      <c r="I11" s="43">
+        <f>'TOTAL RH'!I4</f>
+        <v/>
+      </c>
       <c r="J11" s="43">
-        <f>'TOTAL RH'!I4</f>
-        <v/>
-      </c>
-      <c r="K11" s="43">
         <f>'TOTAL RH'!J4</f>
         <v/>
       </c>
+      <c r="K11" s="1" t="n"/>
       <c r="L11" s="1" t="n"/>
       <c r="M11" s="1" t="n"/>
       <c r="N11" s="1" t="n"/>
       <c r="O11" s="1" t="n"/>
       <c r="P11" s="1" t="n"/>
-      <c r="Q11" s="1" t="n"/>
-      <c r="R11" s="1" t="n"/>
-      <c r="S11" s="1" t="n"/>
-      <c r="T11" s="1" t="n"/>
     </row>
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="1" t="n"/>
@@ -7479,29 +7442,25 @@
       <c r="E12" s="1" t="n"/>
       <c r="F12" s="1" t="n"/>
       <c r="G12" s="1" t="n"/>
-      <c r="H12" s="1" t="n"/>
-      <c r="I12" s="44" t="inlineStr">
+      <c r="H12" s="44" t="inlineStr">
         <is>
           <t>Booking Pending pick up</t>
         </is>
       </c>
+      <c r="I12" s="45">
+        <f>'TOTAL RH'!I5</f>
+        <v/>
+      </c>
       <c r="J12" s="45">
-        <f>'TOTAL RH'!I5</f>
-        <v/>
-      </c>
-      <c r="K12" s="45">
         <f>'TOTAL RH'!J5</f>
         <v/>
       </c>
+      <c r="K12" s="1" t="n"/>
       <c r="L12" s="1" t="n"/>
       <c r="M12" s="1" t="n"/>
       <c r="N12" s="1" t="n"/>
       <c r="O12" s="1" t="n"/>
       <c r="P12" s="1" t="n"/>
-      <c r="Q12" s="1" t="n"/>
-      <c r="R12" s="1" t="n"/>
-      <c r="S12" s="1" t="n"/>
-      <c r="T12" s="1" t="n"/>
     </row>
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="1" t="n"/>
@@ -7521,29 +7480,25 @@
       <c r="E13" s="1" t="n"/>
       <c r="F13" s="1" t="n"/>
       <c r="G13" s="1" t="n"/>
-      <c r="H13" s="1" t="n"/>
-      <c r="I13" s="44" t="inlineStr">
+      <c r="H13" s="44" t="inlineStr">
         <is>
           <t>Booking on today</t>
         </is>
       </c>
+      <c r="I13" s="45">
+        <f>'TOTAL RH'!I6</f>
+        <v/>
+      </c>
       <c r="J13" s="45">
-        <f>'TOTAL RH'!I6</f>
-        <v/>
-      </c>
-      <c r="K13" s="45">
         <f>'TOTAL RH'!J6</f>
         <v/>
       </c>
+      <c r="K13" s="1" t="n"/>
       <c r="L13" s="1" t="n"/>
       <c r="M13" s="1" t="n"/>
       <c r="N13" s="1" t="n"/>
       <c r="O13" s="1" t="n"/>
       <c r="P13" s="1" t="n"/>
-      <c r="Q13" s="1" t="n"/>
-      <c r="R13" s="1" t="n"/>
-      <c r="S13" s="1" t="n"/>
-      <c r="T13" s="1" t="n"/>
     </row>
     <row r="14" ht="13" customHeight="1">
       <c r="A14" s="1" t="n"/>
@@ -7563,29 +7518,25 @@
       <c r="E14" s="1" t="n"/>
       <c r="F14" s="1" t="n"/>
       <c r="G14" s="1" t="n"/>
-      <c r="H14" s="1" t="n"/>
-      <c r="I14" s="44" t="inlineStr">
+      <c r="H14" s="44" t="inlineStr">
         <is>
           <t>Booking rest of this week</t>
         </is>
       </c>
+      <c r="I14" s="45">
+        <f>'TOTAL RH'!I7</f>
+        <v/>
+      </c>
       <c r="J14" s="45">
-        <f>'TOTAL RH'!I7</f>
-        <v/>
-      </c>
-      <c r="K14" s="45">
         <f>'TOTAL RH'!J7</f>
         <v/>
       </c>
+      <c r="K14" s="1" t="n"/>
       <c r="L14" s="1" t="n"/>
       <c r="M14" s="1" t="n"/>
       <c r="N14" s="1" t="n"/>
       <c r="O14" s="1" t="n"/>
       <c r="P14" s="1" t="n"/>
-      <c r="Q14" s="1" t="n"/>
-      <c r="R14" s="1" t="n"/>
-      <c r="S14" s="1" t="n"/>
-      <c r="T14" s="1" t="n"/>
     </row>
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="1" t="n"/>
@@ -7605,29 +7556,25 @@
       <c r="E15" s="1" t="n"/>
       <c r="F15" s="1" t="n"/>
       <c r="G15" s="1" t="n"/>
-      <c r="H15" s="1" t="n"/>
-      <c r="I15" s="46" t="inlineStr">
+      <c r="H15" s="46" t="inlineStr">
         <is>
           <t>AV Balance till 19 SEP</t>
         </is>
       </c>
+      <c r="I15" s="47">
+        <f>'TOTAL RH'!I8</f>
+        <v/>
+      </c>
       <c r="J15" s="47">
-        <f>'TOTAL RH'!I8</f>
-        <v/>
-      </c>
-      <c r="K15" s="47">
         <f>'TOTAL RH'!J8</f>
         <v/>
       </c>
+      <c r="K15" s="1" t="n"/>
       <c r="L15" s="1" t="n"/>
       <c r="M15" s="1" t="n"/>
       <c r="N15" s="1" t="n"/>
       <c r="O15" s="1" t="n"/>
       <c r="P15" s="1" t="n"/>
-      <c r="Q15" s="1" t="n"/>
-      <c r="R15" s="1" t="n"/>
-      <c r="S15" s="1" t="n"/>
-      <c r="T15" s="1" t="n"/>
     </row>
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="1" t="n"/>
@@ -7647,29 +7594,25 @@
       <c r="E16" s="1" t="n"/>
       <c r="F16" s="1" t="n"/>
       <c r="G16" s="1" t="n"/>
-      <c r="H16" s="1" t="n"/>
-      <c r="I16" s="44" t="inlineStr">
+      <c r="H16" s="44" t="inlineStr">
         <is>
           <t>Booking 21-26 SEP</t>
         </is>
       </c>
+      <c r="I16" s="45">
+        <f>'TOTAL RH'!I9</f>
+        <v/>
+      </c>
       <c r="J16" s="45">
-        <f>'TOTAL RH'!I9</f>
-        <v/>
-      </c>
-      <c r="K16" s="45">
         <f>'TOTAL RH'!J9</f>
         <v/>
       </c>
+      <c r="K16" s="1" t="n"/>
       <c r="L16" s="1" t="n"/>
       <c r="M16" s="1" t="n"/>
       <c r="N16" s="1" t="n"/>
       <c r="O16" s="1" t="n"/>
       <c r="P16" s="1" t="n"/>
-      <c r="Q16" s="1" t="n"/>
-      <c r="R16" s="1" t="n"/>
-      <c r="S16" s="1" t="n"/>
-      <c r="T16" s="1" t="n"/>
     </row>
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="1" t="n"/>
@@ -7689,29 +7632,25 @@
       <c r="E17" s="1" t="n"/>
       <c r="F17" s="1" t="n"/>
       <c r="G17" s="1" t="n"/>
-      <c r="H17" s="1" t="n"/>
-      <c r="I17" s="46" t="inlineStr">
+      <c r="H17" s="46" t="inlineStr">
         <is>
           <t>AV Balance till 26 SEP</t>
         </is>
       </c>
+      <c r="I17" s="47">
+        <f>'TOTAL RH'!I10</f>
+        <v/>
+      </c>
       <c r="J17" s="47">
-        <f>'TOTAL RH'!I10</f>
-        <v/>
-      </c>
-      <c r="K17" s="47">
         <f>'TOTAL RH'!J10</f>
         <v/>
       </c>
+      <c r="K17" s="1" t="n"/>
       <c r="L17" s="1" t="n"/>
       <c r="M17" s="1" t="n"/>
       <c r="N17" s="1" t="n"/>
       <c r="O17" s="1" t="n"/>
       <c r="P17" s="1" t="n"/>
-      <c r="Q17" s="1" t="n"/>
-      <c r="R17" s="1" t="n"/>
-      <c r="S17" s="1" t="n"/>
-      <c r="T17" s="1" t="n"/>
     </row>
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="1" t="n"/>
@@ -7731,29 +7670,25 @@
       <c r="E18" s="1" t="n"/>
       <c r="F18" s="1" t="n"/>
       <c r="G18" s="1" t="n"/>
-      <c r="H18" s="1" t="n"/>
-      <c r="I18" s="44" t="inlineStr">
+      <c r="H18" s="44" t="inlineStr">
         <is>
           <t>Booking 28 SEP-3 OCT</t>
         </is>
       </c>
+      <c r="I18" s="45">
+        <f>'TOTAL RH'!I11</f>
+        <v/>
+      </c>
       <c r="J18" s="45">
-        <f>'TOTAL RH'!I11</f>
-        <v/>
-      </c>
-      <c r="K18" s="45">
         <f>'TOTAL RH'!J11</f>
         <v/>
       </c>
+      <c r="K18" s="1" t="n"/>
       <c r="L18" s="1" t="n"/>
       <c r="M18" s="1" t="n"/>
       <c r="N18" s="1" t="n"/>
       <c r="O18" s="1" t="n"/>
       <c r="P18" s="1" t="n"/>
-      <c r="Q18" s="1" t="n"/>
-      <c r="R18" s="1" t="n"/>
-      <c r="S18" s="1" t="n"/>
-      <c r="T18" s="1" t="n"/>
     </row>
     <row r="19" ht="13" customHeight="1">
       <c r="A19" s="1" t="n"/>
@@ -7773,29 +7708,25 @@
       <c r="E19" s="1" t="n"/>
       <c r="F19" s="1" t="n"/>
       <c r="G19" s="1" t="n"/>
-      <c r="H19" s="1" t="n"/>
-      <c r="I19" s="46" t="inlineStr">
+      <c r="H19" s="46" t="inlineStr">
         <is>
           <t>AV Balance till 3 OCT</t>
         </is>
       </c>
-      <c r="J19" s="47">
+      <c r="I19" s="47">
         <f>'TOTAL RH'!I12</f>
         <v/>
       </c>
-      <c r="K19" s="55">
+      <c r="J19" s="55">
         <f>'TOTAL RH'!J12</f>
         <v/>
       </c>
+      <c r="K19" s="1" t="n"/>
       <c r="L19" s="1" t="n"/>
       <c r="M19" s="1" t="n"/>
       <c r="N19" s="1" t="n"/>
       <c r="O19" s="1" t="n"/>
       <c r="P19" s="1" t="n"/>
-      <c r="Q19" s="1" t="n"/>
-      <c r="R19" s="1" t="n"/>
-      <c r="S19" s="1" t="n"/>
-      <c r="T19" s="1" t="n"/>
     </row>
     <row r="20" ht="13" customHeight="1">
       <c r="A20" s="1" t="n"/>
@@ -7814,10 +7745,6 @@
       <c r="N20" s="1" t="n"/>
       <c r="O20" s="1" t="n"/>
       <c r="P20" s="1" t="n"/>
-      <c r="Q20" s="1" t="n"/>
-      <c r="R20" s="1" t="n"/>
-      <c r="S20" s="1" t="n"/>
-      <c r="T20" s="1" t="n"/>
     </row>
     <row r="21" ht="13" customHeight="1">
       <c r="A21" s="1" t="n"/>
@@ -7836,10 +7763,6 @@
       <c r="N21" s="1" t="n"/>
       <c r="O21" s="1" t="n"/>
       <c r="P21" s="1" t="n"/>
-      <c r="Q21" s="1" t="n"/>
-      <c r="R21" s="1" t="n"/>
-      <c r="S21" s="1" t="n"/>
-      <c r="T21" s="1" t="n"/>
     </row>
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="1" t="n"/>
@@ -7862,10 +7785,6 @@
       <c r="N22" s="1" t="n"/>
       <c r="O22" s="1" t="n"/>
       <c r="P22" s="1" t="n"/>
-      <c r="Q22" s="1" t="n"/>
-      <c r="R22" s="1" t="n"/>
-      <c r="S22" s="1" t="n"/>
-      <c r="T22" s="1" t="n"/>
     </row>
     <row r="23" ht="13" customHeight="1">
       <c r="A23" s="1" t="n"/>
@@ -7878,22 +7797,18 @@
       <c r="E23" s="1" t="n"/>
       <c r="F23" s="1" t="n"/>
       <c r="G23" s="1" t="n"/>
-      <c r="H23" s="1" t="n"/>
-      <c r="I23" s="40">
+      <c r="H23" s="40">
         <f>'TOTAL RH'!H2</f>
         <v/>
       </c>
-      <c r="J23" s="53" t="n"/>
-      <c r="K23" s="54" t="n"/>
+      <c r="I23" s="53" t="n"/>
+      <c r="J23" s="54" t="n"/>
+      <c r="K23" s="1" t="n"/>
       <c r="L23" s="1" t="n"/>
       <c r="M23" s="1" t="n"/>
       <c r="N23" s="1" t="n"/>
       <c r="O23" s="1" t="n"/>
       <c r="P23" s="1" t="n"/>
-      <c r="Q23" s="1" t="n"/>
-      <c r="R23" s="1" t="n"/>
-      <c r="S23" s="1" t="n"/>
-      <c r="T23" s="1" t="n"/>
     </row>
     <row r="24" ht="13" customHeight="1">
       <c r="A24" s="1" t="n"/>
@@ -7911,27 +7826,23 @@
       <c r="E24" s="1" t="n"/>
       <c r="F24" s="1" t="n"/>
       <c r="G24" s="1" t="n"/>
-      <c r="H24" s="1" t="n"/>
-      <c r="I24" s="34" t="n"/>
+      <c r="H24" s="34" t="n"/>
+      <c r="I24" s="41" t="inlineStr">
+        <is>
+          <t>20'RE</t>
+        </is>
+      </c>
       <c r="J24" s="41" t="inlineStr">
         <is>
-          <t>20'RE</t>
-        </is>
-      </c>
-      <c r="K24" s="41" t="inlineStr">
-        <is>
           <t>40'RH</t>
         </is>
       </c>
+      <c r="K24" s="1" t="n"/>
       <c r="L24" s="1" t="n"/>
       <c r="M24" s="1" t="n"/>
       <c r="N24" s="1" t="n"/>
       <c r="O24" s="1" t="n"/>
       <c r="P24" s="1" t="n"/>
-      <c r="Q24" s="1" t="n"/>
-      <c r="R24" s="1" t="n"/>
-      <c r="S24" s="1" t="n"/>
-      <c r="T24" s="1" t="n"/>
     </row>
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="1" t="n"/>
@@ -7951,29 +7862,25 @@
       <c r="E25" s="1" t="n"/>
       <c r="F25" s="1" t="n"/>
       <c r="G25" s="1" t="n"/>
-      <c r="H25" s="1" t="n"/>
-      <c r="I25" s="34" t="inlineStr">
+      <c r="H25" s="34" t="inlineStr">
         <is>
           <t>AV</t>
         </is>
       </c>
+      <c r="I25" s="45">
+        <f>'TOTAL RH'!I16</f>
+        <v/>
+      </c>
       <c r="J25" s="45">
-        <f>'TOTAL RH'!I16</f>
-        <v/>
-      </c>
-      <c r="K25" s="45">
         <f>'TOTAL RH'!J16</f>
         <v/>
       </c>
+      <c r="K25" s="1" t="n"/>
       <c r="L25" s="1" t="n"/>
       <c r="M25" s="1" t="n"/>
       <c r="N25" s="1" t="n"/>
       <c r="O25" s="1" t="n"/>
       <c r="P25" s="1" t="n"/>
-      <c r="Q25" s="1" t="n"/>
-      <c r="R25" s="1" t="n"/>
-      <c r="S25" s="1" t="n"/>
-      <c r="T25" s="1" t="n"/>
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="1" t="n"/>
@@ -7993,29 +7900,25 @@
       <c r="E26" s="1" t="n"/>
       <c r="F26" s="1" t="n"/>
       <c r="G26" s="1" t="n"/>
-      <c r="H26" s="1" t="n"/>
-      <c r="I26" s="34" t="inlineStr">
+      <c r="H26" s="34" t="inlineStr">
         <is>
           <t>DMG</t>
         </is>
       </c>
+      <c r="I26" s="45">
+        <f>'TOTAL RH'!I17</f>
+        <v/>
+      </c>
       <c r="J26" s="45">
-        <f>'TOTAL RH'!I17</f>
-        <v/>
-      </c>
-      <c r="K26" s="45">
         <f>'TOTAL RH'!J17</f>
         <v/>
       </c>
+      <c r="K26" s="1" t="n"/>
       <c r="L26" s="1" t="n"/>
       <c r="M26" s="1" t="n"/>
       <c r="N26" s="1" t="n"/>
       <c r="O26" s="1" t="n"/>
       <c r="P26" s="1" t="n"/>
-      <c r="Q26" s="1" t="n"/>
-      <c r="R26" s="1" t="n"/>
-      <c r="S26" s="1" t="n"/>
-      <c r="T26" s="1" t="n"/>
     </row>
     <row r="27" ht="13" customHeight="1">
       <c r="A27" s="1" t="n"/>
@@ -8034,10 +7937,6 @@
       <c r="N27" s="1" t="n"/>
       <c r="O27" s="1" t="n"/>
       <c r="P27" s="1" t="n"/>
-      <c r="Q27" s="1" t="n"/>
-      <c r="R27" s="1" t="n"/>
-      <c r="S27" s="1" t="n"/>
-      <c r="T27" s="1" t="n"/>
     </row>
     <row r="28" ht="13" customHeight="1">
       <c r="A28" s="1" t="n"/>
@@ -8056,10 +7955,6 @@
       <c r="N28" s="1" t="n"/>
       <c r="O28" s="1" t="n"/>
       <c r="P28" s="1" t="n"/>
-      <c r="Q28" s="1" t="n"/>
-      <c r="R28" s="1" t="n"/>
-      <c r="S28" s="1" t="n"/>
-      <c r="T28" s="1" t="n"/>
     </row>
     <row r="29" ht="13" customHeight="1">
       <c r="A29" s="1" t="n"/>
@@ -8082,10 +7977,6 @@
       <c r="N29" s="1" t="n"/>
       <c r="O29" s="1" t="n"/>
       <c r="P29" s="1" t="n"/>
-      <c r="Q29" s="1" t="n"/>
-      <c r="R29" s="1" t="n"/>
-      <c r="S29" s="1" t="n"/>
-      <c r="T29" s="1" t="n"/>
     </row>
     <row r="30" ht="13" customHeight="1">
       <c r="A30" s="1" t="n"/>
@@ -8094,32 +7985,28 @@
           <t>BKK27 2020-26 BUILT</t>
         </is>
       </c>
-      <c r="C30" s="53" t="n"/>
-      <c r="D30" s="53" t="n"/>
-      <c r="E30" s="54" t="n"/>
-      <c r="F30" s="1" t="n"/>
-      <c r="G30" s="33" t="inlineStr">
+      <c r="C30" s="34" t="n"/>
+      <c r="D30" s="34" t="n"/>
+      <c r="E30" s="1" t="n"/>
+      <c r="F30" s="33" t="inlineStr">
         <is>
           <t>LCH27 2020-26 BUILT</t>
         </is>
       </c>
-      <c r="H30" s="53" t="n"/>
-      <c r="I30" s="53" t="n"/>
-      <c r="J30" s="54" t="n"/>
-      <c r="K30" s="1" t="n"/>
-      <c r="L30" s="33" t="inlineStr">
+      <c r="G30" s="34" t="n"/>
+      <c r="H30" s="34" t="n"/>
+      <c r="I30" s="1" t="n"/>
+      <c r="J30" s="33" t="inlineStr">
         <is>
           <t>PEAK BUILD YEAR</t>
         </is>
       </c>
-      <c r="M30" s="53" t="n"/>
-      <c r="N30" s="53" t="n"/>
-      <c r="O30" s="54" t="n"/>
+      <c r="K30" s="34" t="n"/>
+      <c r="L30" s="34" t="n"/>
+      <c r="M30" s="1" t="n"/>
+      <c r="N30" s="1" t="n"/>
+      <c r="O30" s="1" t="n"/>
       <c r="P30" s="1" t="n"/>
-      <c r="Q30" s="1" t="n"/>
-      <c r="R30" s="1" t="n"/>
-      <c r="S30" s="1" t="n"/>
-      <c r="T30" s="1" t="n"/>
     </row>
     <row r="31" ht="13" customHeight="1">
       <c r="A31" s="1" t="n"/>
@@ -8127,30 +8014,26 @@
         <f>SUM('TOTAL RH'!D36:D42)+SUM('TOTAL RH'!F36:F42)+SUM('TOTAL RH'!H36:H42)</f>
         <v/>
       </c>
-      <c r="C31" s="53" t="n"/>
-      <c r="D31" s="53" t="n"/>
-      <c r="E31" s="54" t="n"/>
-      <c r="F31" s="1" t="n"/>
-      <c r="G31" s="49">
+      <c r="C31" s="34" t="n"/>
+      <c r="D31" s="34" t="n"/>
+      <c r="E31" s="1" t="n"/>
+      <c r="F31" s="49">
         <f>SUM('TOTAL RH'!L36:L42)+SUM('TOTAL RH'!N36:N42)+SUM('TOTAL RH'!P36:P42)</f>
         <v/>
       </c>
-      <c r="H31" s="53" t="n"/>
-      <c r="I31" s="53" t="n"/>
-      <c r="J31" s="54" t="n"/>
-      <c r="K31" s="1" t="n"/>
-      <c r="L31" s="36">
+      <c r="G31" s="34" t="n"/>
+      <c r="H31" s="34" t="n"/>
+      <c r="I31" s="1" t="n"/>
+      <c r="J31" s="36">
         <f>"2021 / 2019"</f>
         <v/>
       </c>
-      <c r="M31" s="53" t="n"/>
-      <c r="N31" s="53" t="n"/>
-      <c r="O31" s="54" t="n"/>
+      <c r="K31" s="34" t="n"/>
+      <c r="L31" s="34" t="n"/>
+      <c r="M31" s="1" t="n"/>
+      <c r="N31" s="1" t="n"/>
+      <c r="O31" s="1" t="n"/>
       <c r="P31" s="1" t="n"/>
-      <c r="Q31" s="1" t="n"/>
-      <c r="R31" s="1" t="n"/>
-      <c r="S31" s="1" t="n"/>
-      <c r="T31" s="1" t="n"/>
     </row>
     <row r="32" ht="13" customHeight="1">
       <c r="A32" s="1" t="n"/>
@@ -8159,32 +8042,28 @@
           <t>of 40'RH on hand</t>
         </is>
       </c>
-      <c r="C32" s="53" t="n"/>
-      <c r="D32" s="53" t="n"/>
-      <c r="E32" s="54" t="n"/>
-      <c r="F32" s="1" t="n"/>
-      <c r="G32" s="37" t="inlineStr">
+      <c r="C32" s="34" t="n"/>
+      <c r="D32" s="34" t="n"/>
+      <c r="E32" s="1" t="n"/>
+      <c r="F32" s="37" t="inlineStr">
         <is>
           <t>of 40'RH on hand</t>
         </is>
       </c>
-      <c r="H32" s="53" t="n"/>
-      <c r="I32" s="53" t="n"/>
-      <c r="J32" s="54" t="n"/>
-      <c r="K32" s="1" t="n"/>
-      <c r="L32" s="37" t="inlineStr">
+      <c r="G32" s="34" t="n"/>
+      <c r="H32" s="34" t="n"/>
+      <c r="I32" s="1" t="n"/>
+      <c r="J32" s="37" t="inlineStr">
         <is>
           <t>19 units across both depots</t>
         </is>
       </c>
-      <c r="M32" s="53" t="n"/>
-      <c r="N32" s="53" t="n"/>
-      <c r="O32" s="54" t="n"/>
+      <c r="K32" s="34" t="n"/>
+      <c r="L32" s="34" t="n"/>
+      <c r="M32" s="1" t="n"/>
+      <c r="N32" s="1" t="n"/>
+      <c r="O32" s="1" t="n"/>
       <c r="P32" s="1" t="n"/>
-      <c r="Q32" s="1" t="n"/>
-      <c r="R32" s="1" t="n"/>
-      <c r="S32" s="1" t="n"/>
-      <c r="T32" s="1" t="n"/>
     </row>
     <row r="33" ht="13" customHeight="1">
       <c r="A33" s="1" t="n"/>
@@ -8203,10 +8082,6 @@
       <c r="N33" s="1" t="n"/>
       <c r="O33" s="1" t="n"/>
       <c r="P33" s="1" t="n"/>
-      <c r="Q33" s="1" t="n"/>
-      <c r="R33" s="1" t="n"/>
-      <c r="S33" s="1" t="n"/>
-      <c r="T33" s="1" t="n"/>
     </row>
     <row r="34" ht="13" customHeight="1">
       <c r="A34" s="1" t="n"/>
@@ -8220,23 +8095,19 @@
       <c r="E34" s="1" t="n"/>
       <c r="F34" s="1" t="n"/>
       <c r="G34" s="1" t="n"/>
-      <c r="H34" s="1" t="n"/>
-      <c r="I34" s="40" t="inlineStr">
+      <c r="H34" s="40" t="inlineStr">
         <is>
           <t>LCH27 current mix</t>
         </is>
       </c>
-      <c r="J34" s="53" t="n"/>
-      <c r="K34" s="54" t="n"/>
+      <c r="I34" s="53" t="n"/>
+      <c r="J34" s="54" t="n"/>
+      <c r="K34" s="1" t="n"/>
       <c r="L34" s="1" t="n"/>
       <c r="M34" s="1" t="n"/>
       <c r="N34" s="1" t="n"/>
       <c r="O34" s="1" t="n"/>
       <c r="P34" s="1" t="n"/>
-      <c r="Q34" s="1" t="n"/>
-      <c r="R34" s="1" t="n"/>
-      <c r="S34" s="1" t="n"/>
-      <c r="T34" s="1" t="n"/>
     </row>
     <row r="35" ht="13" customHeight="1">
       <c r="A35" s="1" t="n"/>
@@ -8254,27 +8125,23 @@
       <c r="E35" s="1" t="n"/>
       <c r="F35" s="1" t="n"/>
       <c r="G35" s="1" t="n"/>
-      <c r="H35" s="1" t="n"/>
-      <c r="I35" s="34" t="n"/>
+      <c r="H35" s="34" t="n"/>
+      <c r="I35" s="41" t="inlineStr">
+        <is>
+          <t>22RE</t>
+        </is>
+      </c>
       <c r="J35" s="41" t="inlineStr">
         <is>
-          <t>22RE</t>
-        </is>
-      </c>
-      <c r="K35" s="41" t="inlineStr">
-        <is>
-          <t>45RE</t>
-        </is>
-      </c>
+          <t>45RE</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="n"/>
       <c r="L35" s="1" t="n"/>
       <c r="M35" s="1" t="n"/>
       <c r="N35" s="1" t="n"/>
       <c r="O35" s="1" t="n"/>
       <c r="P35" s="1" t="n"/>
-      <c r="Q35" s="1" t="n"/>
-      <c r="R35" s="1" t="n"/>
-      <c r="S35" s="1" t="n"/>
-      <c r="T35" s="1" t="n"/>
     </row>
     <row r="36" ht="13" customHeight="1">
       <c r="A36" s="1" t="n"/>
@@ -8294,29 +8161,25 @@
       <c r="E36" s="1" t="n"/>
       <c r="F36" s="1" t="n"/>
       <c r="G36" s="1" t="n"/>
-      <c r="H36" s="1" t="n"/>
-      <c r="I36" s="34" t="inlineStr">
+      <c r="H36" s="34" t="inlineStr">
         <is>
           <t>CARRIER</t>
         </is>
       </c>
+      <c r="I36" s="45">
+        <f>'TOTAL RH'!K53</f>
+        <v/>
+      </c>
       <c r="J36" s="45">
-        <f>'TOTAL RH'!K53</f>
-        <v/>
-      </c>
-      <c r="K36" s="45">
         <f>'TOTAL RH'!L53</f>
         <v/>
       </c>
+      <c r="K36" s="1" t="n"/>
       <c r="L36" s="1" t="n"/>
       <c r="M36" s="1" t="n"/>
       <c r="N36" s="1" t="n"/>
       <c r="O36" s="1" t="n"/>
       <c r="P36" s="1" t="n"/>
-      <c r="Q36" s="1" t="n"/>
-      <c r="R36" s="1" t="n"/>
-      <c r="S36" s="1" t="n"/>
-      <c r="T36" s="1" t="n"/>
     </row>
     <row r="37" ht="13" customHeight="1">
       <c r="A37" s="1" t="n"/>
@@ -8336,29 +8199,25 @@
       <c r="E37" s="1" t="n"/>
       <c r="F37" s="1" t="n"/>
       <c r="G37" s="1" t="n"/>
-      <c r="H37" s="1" t="n"/>
-      <c r="I37" s="34" t="inlineStr">
+      <c r="H37" s="34" t="inlineStr">
         <is>
           <t>DAIKIN</t>
         </is>
       </c>
+      <c r="I37" s="45">
+        <f>'TOTAL RH'!M53</f>
+        <v/>
+      </c>
       <c r="J37" s="45">
-        <f>'TOTAL RH'!M53</f>
-        <v/>
-      </c>
-      <c r="K37" s="45">
         <f>'TOTAL RH'!N53</f>
         <v/>
       </c>
+      <c r="K37" s="1" t="n"/>
       <c r="L37" s="1" t="n"/>
       <c r="M37" s="1" t="n"/>
       <c r="N37" s="1" t="n"/>
       <c r="O37" s="1" t="n"/>
       <c r="P37" s="1" t="n"/>
-      <c r="Q37" s="1" t="n"/>
-      <c r="R37" s="1" t="n"/>
-      <c r="S37" s="1" t="n"/>
-      <c r="T37" s="1" t="n"/>
     </row>
     <row r="38" ht="13" customHeight="1">
       <c r="A38" s="1" t="n"/>
@@ -8378,29 +8237,25 @@
       <c r="E38" s="1" t="n"/>
       <c r="F38" s="1" t="n"/>
       <c r="G38" s="1" t="n"/>
-      <c r="H38" s="1" t="n"/>
-      <c r="I38" s="34" t="inlineStr">
+      <c r="H38" s="34" t="inlineStr">
         <is>
           <t>THERMO KING</t>
         </is>
       </c>
+      <c r="I38" s="45">
+        <f>'TOTAL RH'!O53</f>
+        <v/>
+      </c>
       <c r="J38" s="45">
-        <f>'TOTAL RH'!O53</f>
-        <v/>
-      </c>
-      <c r="K38" s="45">
         <f>'TOTAL RH'!P53</f>
         <v/>
       </c>
+      <c r="K38" s="1" t="n"/>
       <c r="L38" s="1" t="n"/>
       <c r="M38" s="1" t="n"/>
       <c r="N38" s="1" t="n"/>
       <c r="O38" s="1" t="n"/>
       <c r="P38" s="1" t="n"/>
-      <c r="Q38" s="1" t="n"/>
-      <c r="R38" s="1" t="n"/>
-      <c r="S38" s="1" t="n"/>
-      <c r="T38" s="1" t="n"/>
     </row>
     <row r="39" ht="13" customHeight="1">
       <c r="A39" s="1" t="n"/>
@@ -8419,10 +8274,6 @@
       <c r="N39" s="1" t="n"/>
       <c r="O39" s="1" t="n"/>
       <c r="P39" s="1" t="n"/>
-      <c r="Q39" s="1" t="n"/>
-      <c r="R39" s="1" t="n"/>
-      <c r="S39" s="1" t="n"/>
-      <c r="T39" s="1" t="n"/>
     </row>
     <row r="40" ht="13" customHeight="1">
       <c r="A40" s="1" t="n"/>
@@ -8445,41 +8296,16 @@
       <c r="N40" s="1" t="n"/>
       <c r="O40" s="1" t="n"/>
       <c r="P40" s="1" t="n"/>
-      <c r="Q40" s="1" t="n"/>
-      <c r="R40" s="1" t="n"/>
-      <c r="S40" s="1" t="n"/>
-      <c r="T40" s="1" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="L31:O31"/>
+  <mergeCells count="7">
+    <mergeCell ref="B1:P2"/>
     <mergeCell ref="B23:D23"/>
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="H9:J9"/>
     <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="I23:K23"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="L32:O32"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="I34:K34"/>
-    <mergeCell ref="Q5:T5"/>
-    <mergeCell ref="L5:O5"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="Q4:T4"/>
-    <mergeCell ref="L30:O30"/>
-    <mergeCell ref="B1:S2"/>
-    <mergeCell ref="L4:O4"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="Q6:T6"/>
-    <mergeCell ref="G5:J5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>